<commit_message>
Import Inventory Report 20260701
</commit_message>
<xml_diff>
--- a/reports/Import PO Status.xlsx
+++ b/reports/Import PO Status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP ProBook 455 G10\Documents\1. 일룸구매팀 업무\14_2. Import Inventory Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB1D56FC-0C5A-4B08-A9DF-34F3FB3FEDC8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F31D71-8591-43EE-9AC5-84315333F61F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12135" activeTab="1" xr2:uid="{CDEF7A78-96F0-4F9B-A2AE-3DAFCFC574C3}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12135" xr2:uid="{CDEF7A78-96F0-4F9B-A2AE-3DAFCFC574C3}"/>
   </bookViews>
   <sheets>
     <sheet name="PO피벗" sheetId="4" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId4"/>
+    <pivotCache cacheId="10" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="111">
   <si>
     <t>PO issue date</t>
   </si>
@@ -380,6 +380,14 @@
     <t>ILL10DE00A-L851A</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>HCH9003-3J3CZ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ITY00AG01A-BNT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -491,7 +499,31 @@
     <cellStyle name="표준" xfId="0" builtinId="0"/>
     <cellStyle name="표준 2" xfId="2" xr:uid="{1BC0D383-C5B5-4841-B65D-9934AA451E44}"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="16">
+    <dxf>
+      <numFmt numFmtId="177" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="177" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="177" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="177" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="177" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="177" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="177" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="177" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="177" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
     </dxf>
@@ -530,7 +562,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="LukeBae" refreshedDate="46202.405728587961" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="628" xr:uid="{16FDB7BC-6348-4F2A-AE83-CDA0CBEDCF91}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="LukeBae" refreshedDate="46203.656412037039" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="628" xr:uid="{16FDB7BC-6348-4F2A-AE83-CDA0CBEDCF91}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:K10000" sheet="PO현황"/>
   </cacheSource>
@@ -745,7 +777,7 @@
     <m/>
     <n v="49"/>
     <n v="1.6333333333333333"/>
-    <x v="1"/>
+    <x v="0"/>
   </r>
   <r>
     <x v="0"/>
@@ -758,7 +790,7 @@
     <m/>
     <n v="49"/>
     <n v="1.6333333333333333"/>
-    <x v="1"/>
+    <x v="0"/>
   </r>
   <r>
     <x v="0"/>
@@ -771,7 +803,7 @@
     <m/>
     <n v="49"/>
     <n v="1.6333333333333333"/>
-    <x v="1"/>
+    <x v="0"/>
   </r>
   <r>
     <x v="0"/>
@@ -784,7 +816,7 @@
     <m/>
     <n v="49"/>
     <n v="1.6333333333333333"/>
-    <x v="1"/>
+    <x v="0"/>
   </r>
   <r>
     <x v="0"/>
@@ -797,7 +829,7 @@
     <m/>
     <n v="49"/>
     <n v="1.6333333333333333"/>
-    <x v="1"/>
+    <x v="0"/>
   </r>
   <r>
     <x v="0"/>
@@ -1525,7 +1557,7 @@
     <m/>
     <n v="86"/>
     <n v="2.8666666666666667"/>
-    <x v="1"/>
+    <x v="0"/>
   </r>
   <r>
     <x v="3"/>
@@ -8863,8 +8895,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C37205E4-72CA-4DE2-9A3D-2593DEDE93D2}" name="피벗 테이블2" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="값" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="A3:I50" firstHeaderRow="1" firstDataRow="3" firstDataCol="2"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C37205E4-72CA-4DE2-9A3D-2593DEDE93D2}" name="피벗 테이블2" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="값" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A3:I49" firstHeaderRow="1" firstDataRow="3" firstDataCol="2"/>
   <pivotFields count="13">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
       <items count="5">
@@ -8978,16 +9010,13 @@
     <field x="0"/>
     <field x="4"/>
   </rowFields>
-  <rowItems count="45">
+  <rowItems count="44">
     <i>
       <x/>
       <x v="2"/>
     </i>
     <i r="1">
       <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
     </i>
     <i r="1">
       <x v="5"/>
@@ -9152,36 +9181,36 @@
     <dataField name="합계 : QTY" fld="5" baseField="0" baseItem="0" numFmtId="177"/>
   </dataFields>
   <formats count="8">
-    <format dxfId="7">
+    <format dxfId="15">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="14">
       <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="13">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="12">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="10" count="0" defaultSubtotal="1"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="8">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="6" count="6">
@@ -9582,9 +9611,6 @@
       <c r="B6" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="8">
-        <v>50</v>
-      </c>
       <c r="F6" s="8">
         <v>50</v>
       </c>
@@ -9592,7 +9618,7 @@
         <v>250</v>
       </c>
       <c r="I6" s="8">
-        <v>350</v>
+        <v>300</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -9608,85 +9634,85 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="8">
-        <v>50</v>
+        <v>35</v>
+      </c>
+      <c r="C8" s="8">
+        <v>30</v>
+      </c>
+      <c r="G8" s="8">
+        <v>30</v>
       </c>
       <c r="I8" s="8">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="8">
-        <v>30</v>
-      </c>
-      <c r="G9" s="8">
-        <v>30</v>
+        <v>17</v>
+      </c>
+      <c r="D9" s="8">
+        <v>490</v>
       </c>
       <c r="I9" s="8">
-        <v>60</v>
+        <v>490</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="8">
-        <v>505</v>
+        <v>33</v>
+      </c>
+      <c r="C10" s="8">
+        <v>100</v>
+      </c>
+      <c r="F10" s="8">
+        <v>80</v>
       </c>
       <c r="I10" s="8">
-        <v>505</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C11" s="8">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="F11" s="8">
-        <v>80</v>
+        <v>128</v>
+      </c>
+      <c r="G11" s="8">
+        <v>120</v>
       </c>
       <c r="I11" s="8">
-        <v>180</v>
+        <v>368</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="8">
-        <v>120</v>
-      </c>
-      <c r="F12" s="8">
-        <v>128</v>
+        <v>41</v>
       </c>
       <c r="G12" s="8">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="I12" s="8">
-        <v>368</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G13" s="8">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="I13" s="8">
-        <v>10</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G14" s="8">
         <v>50</v>
@@ -9697,276 +9723,270 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G15" s="8">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="I15" s="8">
-        <v>50</v>
+        <v>200</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>46</v>
+        <v>36</v>
+      </c>
+      <c r="C16" s="8">
+        <v>50</v>
       </c>
       <c r="G16" s="8">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="I16" s="8">
-        <v>200</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C17" s="8">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="G17" s="8">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="I17" s="8">
-        <v>100</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="C18" s="8">
         <v>20</v>
       </c>
       <c r="G18" s="8">
-        <v>130</v>
+        <v>40</v>
       </c>
       <c r="I18" s="8">
-        <v>150</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C19" s="8">
         <v>20</v>
       </c>
       <c r="G19" s="8">
+        <v>20</v>
+      </c>
+      <c r="I19" s="8">
         <v>40</v>
-      </c>
-      <c r="I19" s="8">
-        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>55</v>
-      </c>
-      <c r="C20" s="8">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="G20" s="8">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="I20" s="8">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G21" s="8">
-        <v>60</v>
+        <v>250</v>
       </c>
       <c r="I21" s="8">
-        <v>60</v>
+        <v>250</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>44</v>
+        <v>38</v>
+      </c>
+      <c r="C22" s="8">
+        <v>70</v>
       </c>
       <c r="G22" s="8">
-        <v>250</v>
+        <v>70</v>
       </c>
       <c r="I22" s="8">
-        <v>250</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C23" s="8">
         <v>70</v>
       </c>
       <c r="G23" s="8">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="I23" s="8">
-        <v>140</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="C24" s="8">
-        <v>70</v>
-      </c>
-      <c r="G24" s="8">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="I24" s="8">
-        <v>220</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="C25" s="8">
-        <v>50</v>
-      </c>
-      <c r="D25" s="8">
         <v>100</v>
       </c>
       <c r="I25" s="8">
-        <v>150</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="C26" s="8">
-        <v>100</v>
+        <v>150</v>
+      </c>
+      <c r="G26" s="8">
+        <v>150</v>
       </c>
       <c r="I26" s="8">
-        <v>100</v>
+        <v>300</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="C27" s="8">
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="G27" s="8">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="I27" s="8">
-        <v>300</v>
+        <v>600</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
-        <v>24</v>
-      </c>
-      <c r="C28" s="8">
-        <v>400</v>
-      </c>
-      <c r="D28" s="8">
         <v>50</v>
       </c>
       <c r="G28" s="8">
+        <v>30</v>
+      </c>
+      <c r="I28" s="8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" t="s">
+        <v>71</v>
+      </c>
+      <c r="G29" s="8">
+        <v>180</v>
+      </c>
+      <c r="I29" s="8">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>69</v>
+      </c>
+      <c r="G30" s="8">
+        <v>190</v>
+      </c>
+      <c r="I30" s="8">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31" t="s">
+        <v>79</v>
+      </c>
+      <c r="H31" s="8">
+        <v>520</v>
+      </c>
+      <c r="I31" s="8">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>80</v>
+      </c>
+      <c r="H32" s="8">
         <v>200</v>
       </c>
-      <c r="I28" s="8">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B29" t="s">
-        <v>50</v>
-      </c>
-      <c r="G29" s="8">
-        <v>30</v>
-      </c>
-      <c r="I29" s="8">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>64</v>
-      </c>
-      <c r="B30" t="s">
-        <v>71</v>
-      </c>
-      <c r="G30" s="8">
-        <v>180</v>
-      </c>
-      <c r="I30" s="8">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B31" t="s">
-        <v>69</v>
-      </c>
-      <c r="G31" s="8">
-        <v>190</v>
-      </c>
-      <c r="I31" s="8">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32" t="s">
-        <v>79</v>
-      </c>
-      <c r="H32" s="8">
-        <v>520</v>
-      </c>
       <c r="I32" s="8">
-        <v>520</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
-        <v>80</v>
-      </c>
-      <c r="H33" s="8">
-        <v>200</v>
+        <v>82</v>
+      </c>
+      <c r="C33" s="8">
+        <v>50</v>
       </c>
       <c r="I33" s="8">
-        <v>200</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>82</v>
-      </c>
-      <c r="C34" s="8">
-        <v>50</v>
+        <v>75</v>
+      </c>
+      <c r="G34" s="8">
+        <v>100</v>
       </c>
       <c r="I34" s="8">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>75</v>
-      </c>
-      <c r="G35" s="8">
-        <v>100</v>
+        <v>76</v>
+      </c>
+      <c r="C35" s="8">
+        <v>50</v>
       </c>
       <c r="I35" s="8">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>76</v>
-      </c>
-      <c r="C36" s="8">
+        <v>77</v>
+      </c>
+      <c r="G36" s="8">
         <v>50</v>
       </c>
       <c r="I36" s="8">
@@ -9975,182 +9995,178 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G37" s="8">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="I37" s="8">
-        <v>50</v>
+        <v>150</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>81</v>
+        <v>78</v>
+      </c>
+      <c r="C38" s="8">
+        <v>300</v>
       </c>
       <c r="G38" s="8">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="I38" s="8">
-        <v>150</v>
+        <v>600</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
       <c r="B39" t="s">
-        <v>78</v>
-      </c>
-      <c r="C39" s="8">
-        <v>300</v>
+        <v>68</v>
+      </c>
+      <c r="E39" s="8">
+        <v>44</v>
       </c>
       <c r="F39" s="8">
-        <v>300</v>
-      </c>
-      <c r="G39" s="8">
-        <v>300</v>
+        <v>44</v>
       </c>
       <c r="I39" s="8">
-        <v>900</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>60</v>
-      </c>
       <c r="B40" t="s">
-        <v>68</v>
-      </c>
-      <c r="E40" s="8">
-        <v>44</v>
-      </c>
-      <c r="F40" s="8">
-        <v>44</v>
+        <v>100</v>
+      </c>
+      <c r="C40" s="8">
+        <v>7</v>
       </c>
       <c r="I40" s="8">
-        <v>88</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C41" s="8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I41" s="8">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C42" s="8">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I42" s="8">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C43" s="8">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="I43" s="8">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C44" s="8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I44" s="8">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C45" s="8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I45" s="8">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C46" s="8">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I46" s="8">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C47" s="8">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="I47" s="8">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>90</v>
+      </c>
       <c r="B48" t="s">
-        <v>107</v>
-      </c>
-      <c r="C48" s="8">
-        <v>6</v>
-      </c>
-      <c r="I48" s="8">
-        <v>6</v>
+        <v>90</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>90</v>
-      </c>
-      <c r="B49" t="s">
-        <v>90</v>
+        <v>91</v>
+      </c>
+      <c r="B49"/>
+      <c r="C49" s="8">
+        <v>1676</v>
+      </c>
+      <c r="D49" s="8">
+        <v>490</v>
+      </c>
+      <c r="E49" s="8">
+        <v>104</v>
+      </c>
+      <c r="F49" s="8">
+        <v>302</v>
+      </c>
+      <c r="G49" s="8">
+        <v>2830</v>
+      </c>
+      <c r="H49" s="8">
+        <v>720</v>
+      </c>
+      <c r="I49" s="8">
+        <v>6122</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>91</v>
-      </c>
       <c r="B50"/>
-      <c r="C50" s="8">
-        <v>1676</v>
-      </c>
-      <c r="D50" s="8">
-        <v>755</v>
-      </c>
-      <c r="E50" s="8">
-        <v>104</v>
-      </c>
-      <c r="F50" s="8">
-        <v>602</v>
-      </c>
-      <c r="G50" s="8">
-        <v>2830</v>
-      </c>
-      <c r="H50" s="8">
-        <v>720</v>
-      </c>
-      <c r="I50" s="8">
-        <v>6687</v>
-      </c>
+      <c r="C50"/>
+      <c r="D50"/>
+      <c r="E50"/>
+      <c r="F50"/>
+      <c r="G50"/>
+      <c r="H50"/>
+      <c r="I50"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -10160,7 +10176,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{402A429B-27CD-4282-8AA6-AA5D0F207858}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:V628"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
@@ -10210,7 +10225,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>59</v>
       </c>
@@ -10336,6 +10351,9 @@
         <f t="shared" si="1"/>
         <v>1.6333333333333333</v>
       </c>
+      <c r="K5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -10367,6 +10385,9 @@
         <f t="shared" si="1"/>
         <v>1.6333333333333333</v>
       </c>
+      <c r="K6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -10382,7 +10403,7 @@
         <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>110</v>
       </c>
       <c r="F7" s="3">
         <v>100</v>
@@ -10398,6 +10419,9 @@
         <f t="shared" si="1"/>
         <v>1.6333333333333333</v>
       </c>
+      <c r="K7" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -10429,6 +10453,9 @@
         <f t="shared" si="1"/>
         <v>1.6333333333333333</v>
       </c>
+      <c r="K8" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -10444,7 +10471,7 @@
         <v>20</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="F9" s="3">
         <v>15</v>
@@ -10460,6 +10487,9 @@
         <f t="shared" si="1"/>
         <v>1.6333333333333333</v>
       </c>
+      <c r="K9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -11989,7 +12019,7 @@
         <v>5.5666666666666664</v>
       </c>
     </row>
-    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>63</v>
       </c>
@@ -12023,7 +12053,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>63</v>
       </c>
@@ -12057,7 +12087,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>63</v>
       </c>
@@ -12091,7 +12121,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="65" spans="1:22" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>63</v>
       </c>
@@ -18004,11 +18034,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K628" xr:uid="{0D65BB20-8C00-496C-AE0F-746BE9424414}">
-    <filterColumn colId="10">
-      <filters blank="1"/>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:K628" xr:uid="{0D65BB20-8C00-496C-AE0F-746BE9424414}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>

</xml_diff>